<commit_message>
Bedakan IABEE GA dari PA pada faktor akreditasi.
Hanya General Accreditation yang disetarakan dengan Internasional. Provisional bukan akreditasi dan memakai peringkat BAN-PT/LAM.

Co-authored-by: m46d45 <m46d45@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/public/Template-Data-PKPRB.xlsx
+++ b/public/Template-Data-PKPRB.xlsx
@@ -267,7 +267,7 @@
     </comment>
     <comment ref="G1" authorId="0" shapeId="0">
       <text>
-        <t>Internasional jika IABEE</t>
+        <t>Internasional hanya untuk IABEE GA. PA memakai peringkat BAN-PT/LAM.</t>
       </text>
     </comment>
     <comment ref="H1" authorId="0" shapeId="0">
@@ -853,7 +853,7 @@
     <row r="22" ht="36" customHeight="1">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>5. IABEE hanya untuk prodi teknik. Jika IABEE general/provisional, akreditasi prodi boleh Internasional.</t>
+          <t>5. IABEE hanya untuk prodi teknik. Hanya IABEE general (GA) yang dicatat sebagai Internasional. Provisional (PA) bukan akreditasi; isi peringkat BAN-PT/LAM dan jangan beri faktor Internasional.</t>
         </is>
       </c>
     </row>
@@ -2076,7 +2076,7 @@
       </c>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>Internasional</t>
+          <t>Unggul</t>
         </is>
       </c>
       <c r="H18" s="6" t="inlineStr">

</xml_diff>

<commit_message>
P1 kuesioner KoNTekS 20: teks, matriks ponsel, kirim aman (#4)
Kuesioner workshop: teks P1, matriks ponsel, kirim idempoten, dan ekspor fasilitator.

IABEE Provisional Accreditation bukan akreditasi. Hanya General Accreditation yang disetarakan dengan Internasional.
</commit_message>
<xml_diff>
--- a/public/Template-Data-PKPRB.xlsx
+++ b/public/Template-Data-PKPRB.xlsx
@@ -267,7 +267,7 @@
     </comment>
     <comment ref="G1" authorId="0" shapeId="0">
       <text>
-        <t>Internasional jika IABEE</t>
+        <t>Internasional hanya untuk IABEE GA. PA memakai peringkat BAN-PT/LAM.</t>
       </text>
     </comment>
     <comment ref="H1" authorId="0" shapeId="0">
@@ -853,7 +853,7 @@
     <row r="22" ht="36" customHeight="1">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>5. IABEE hanya untuk prodi teknik. Jika IABEE general/provisional, akreditasi prodi boleh Internasional.</t>
+          <t>5. IABEE hanya untuk prodi teknik. Hanya IABEE general (GA) yang dicatat sebagai Internasional. Provisional (PA) bukan akreditasi; isi peringkat BAN-PT/LAM dan jangan beri faktor Internasional.</t>
         </is>
       </c>
     </row>
@@ -2076,7 +2076,7 @@
       </c>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>Internasional</t>
+          <t>Unggul</t>
         </is>
       </c>
       <c r="H18" s="6" t="inlineStr">

</xml_diff>